<commit_message>
-copy & paste rooms -area/dims toggle -large room bug fix -'count' column added to input excel - UI colours bug fix
</commit_message>
<xml_diff>
--- a/public/AreaScheduleTemplate.xlsx
+++ b/public/AreaScheduleTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex.macbeth\source\repos\SoAInterface\src\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.macbeth\source\repos\ALMacbeth\Proximate\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC89DC4-78A5-48A6-9B5B-7B9C6A5DFDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B7AD5E-A3ED-41F6-9DCD-07F5C676AD99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{650DD4F8-6989-43F2-8D91-C2298C530FF6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{650DD4F8-6989-43F2-8D91-C2298C530FF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Room Name</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>Example Room A:5,Example Room C:5</t>
+  </si>
+  <si>
+    <t>Count</t>
   </si>
 </sst>
 </file>
@@ -145,12 +148,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{14285DD6-0E0A-4364-AE72-8E546132CD4C}" name="Table1" displayName="Table1" ref="A1:D5" totalsRowShown="0">
-  <autoFilter ref="A1:D5" xr:uid="{14285DD6-0E0A-4364-AE72-8E546132CD4C}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{14285DD6-0E0A-4364-AE72-8E546132CD4C}" name="Table1" displayName="Table1" ref="A1:E5" totalsRowShown="0">
+  <autoFilter ref="A1:E5" xr:uid="{14285DD6-0E0A-4364-AE72-8E546132CD4C}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F2188292-591D-4964-8D61-EA40BCB915F2}" name="Room Name"/>
     <tableColumn id="2" xr3:uid="{BF236702-318B-4AB0-9EB1-A40B4B324E60}" name="Target Area"/>
     <tableColumn id="3" xr3:uid="{A19932EF-4D46-4247-AE69-C4D300233300}" name="Min Width"/>
+    <tableColumn id="5" xr3:uid="{5B1C0BDE-FD63-4337-9EDF-35A96D391E78}" name="Count"/>
     <tableColumn id="4" xr3:uid="{9913EF53-99C4-4220-A973-6FCEB7C3A388}" name="Adjacent Rooms"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -474,17 +478,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB1EB638-892A-49B2-A5C6-E4BC081980DB}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.41796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.68359375" customWidth="1"/>
-    <col min="3" max="3" width="13.15625" customWidth="1"/>
-    <col min="4" max="4" width="35.68359375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.68359375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="4" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -495,21 +499,27 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -519,11 +529,14 @@
       <c r="C3">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -533,16 +546,22 @@
       <c r="C4">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B5">
         <v>15</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>